<commit_message>
chore: commit a stale manual edit to contacts.xlsx
A minor manual change made some time ago that kept showing as an unstaged
modification; committing now only to clear the working tree. No functional
impact on the RDM tooling or docs.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://biomagune-my.sharepoint.com/personal/rtasseff_cicbiomagune_es/Documents/projects/RDM/highCap/gjesus3-pilot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{CDEE3FD6-F154-4441-B7CD-F1C3BDC09426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EACD3C4E-9B0E-486D-AC52-969EFA70D4D2}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{CDEE3FD6-F154-4441-B7CD-F1C3BDC09426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E995F19-E864-5BC3-A12F-7F080C540C6F}"/>
   <bookViews>
-    <workbookView xWindow="9075" yWindow="1860" windowWidth="16740" windowHeight="13170" xr2:uid="{1093DFB4-3B18-4B70-ACD6-0BEA25F3E11E}"/>
+    <workbookView xWindow="2025" yWindow="1140" windowWidth="23940" windowHeight="12870" xr2:uid="{1093DFB4-3B18-4B70-ACD6-0BEA25F3E11E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>